<commit_message>
📊 Horarios actualizados Línea 141 - 4901
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-09-13.xlsx
+++ b/data/horarios-141-2026-09-13.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:11:18</t>
+          <t>Última actualización: 08:54:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>03:11:18</t>
+          <t>08:54:09</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>03:11:18</t>
+          <t>08:54:09</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>04:02</t>
+          <t>09:07</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>51</v>
+        <v>13</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>03:11:18</t>
+          <t>08:54:09</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:48</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>97</v>
+        <v>18</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,23 +548,348 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>03:11:18</t>
+          <t>08:54:09</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>22</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>08:54:09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>23</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>08:54:09</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>09:24</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>30</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>08:54:09</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>40</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>08:54:09</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>41</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>08:54:09</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>102</v>
-      </c>
-      <c r="E9" t="inlineStr">
+      <c r="D14" t="n">
+        <v>51</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>08:54:09</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>09:51</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>57</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>08:54:09</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>61</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>08:54:09</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>70</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>08:54:09</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>76</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>08:54:09</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>81</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>08:54:09</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>10:25</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>91</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>08:54:09</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>100</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>08:54:09</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>110</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -581,7 +906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -594,14 +919,91 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:11:18</t>
+          <t>Última actualización: 08:54:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>08:54:09</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>09:07</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>13</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>08:54:09</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>61</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
         </is>
       </c>
     </row>
@@ -616,7 +1018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -629,14 +1031,166 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:11:18</t>
+          <t>Última actualización: 08:54:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>08:54:09</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>09:03</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>9</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>08:54:09</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>09:28</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>34</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>08:54:09</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>10:18</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>84</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>08:54:09</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>96</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>08:54:09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>109</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>